<commit_message>
Corregge quattro problemi segnalati sull'aggiunta e sull'elenco
- Aggiungi chiede prima il tipo di dispositivo con una tendina, e solo dopo se
  inserirlo a mano o con il lettore: i campi e i codici da leggere seguono il
  tipo scelto, non la schermata da cui si parte.
- Il pulsante Home non riportava all'elenco completo uscendo dal contenitore
  degli iPhone: restava attivo il filtro sul tipo.
- L'elenco parte dal dispositivo piu' recente. Le colonne con una data si
  ordinano per data e non alfabeticamente, e il momento della modifica viene
  registrato al secondo, cosi' due inserimenti ravvicinati restano in ordine.
- Nel contenitore degli iPhone spariscono le colonne del numero di serie e del
  prestito, che per un telefono sono sempre vuote.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Esempio/Inventario.xlsx
+++ b/Esempio/Inventario.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventario" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventario'!$A$1:$M$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventario'!$A$1:$N$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M16"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -440,9 +440,10 @@
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="38" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="38" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,15 +499,20 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>Spedito il</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Ultima modifica</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Modificato da</t>
         </is>
@@ -555,17 +561,18 @@
           <t>30/08/2026 17:00</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
         <is>
           <t>test3</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>30/08/2026 17:00</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>angelotassi@MacBook-Air-di-Angelo.local</t>
         </is>
@@ -615,12 +622,13 @@
         </is>
       </c>
       <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr">
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
         <is>
           <t>30/08/2026 14:58</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>angelotassi@MacBook-Air-di-Angelo.local</t>
         </is>
@@ -661,17 +669,18 @@
       </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
         <is>
           <t>Postazione kiosk 2</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>30/08/2026 14:58</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>angelotassi@MacBook-Air-di-Angelo.local</t>
         </is>
@@ -713,12 +722,13 @@
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr">
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
         <is>
           <t>30/08/2026 14:58</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>angelotassi@MacBook-Air-di-Angelo.local</t>
         </is>
@@ -767,17 +777,18 @@
           <t>30/08/2026 14:58</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
         <is>
           <t>Con custodia rinforzata</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>30/08/2026 14:58</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>angelotassi@MacBook-Air-di-Angelo.local</t>
         </is>
@@ -818,17 +829,18 @@
       </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr">
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
         <is>
           <t>Scorta di emergenza - sigillato</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>30/08/2026 14:58</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>angelotassi@MacBook-Air-di-Angelo.local</t>
         </is>
@@ -869,17 +881,18 @@
       </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr">
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
         <is>
           <t>Scorta di emergenza - sigillato</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>30/08/2026 14:58</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>angelotassi@MacBook-Air-di-Angelo.local</t>
         </is>
@@ -920,17 +933,18 @@
       </c>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr">
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
         <is>
           <t>Kit continuita' operativa</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>30/08/2026 14:58</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>angelotassi@MacBook-Air-di-Angelo.local</t>
         </is>
@@ -971,17 +985,18 @@
       </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr">
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
         <is>
           <t>Postazione kiosk 1</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>30/08/2026 16:13</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>angelotassi@MacBook-Air-di-Angelo.local</t>
         </is>
@@ -990,30 +1005,26 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>7778238723232030230</t>
+          <t>3000003843943</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Iphone</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>7778238723232030230</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Giuseppe sticazzi</t>
-        </is>
-      </c>
+          <t>Lenovo T14 gen 5</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>asdaksjhdkajsdh</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>Site Services BAU</t>
@@ -1021,22 +1032,23 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Disponibile</t>
+          <t>Da rebuildare</t>
         </is>
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>Da rispedire a telefonia</t>
-        </is>
-      </c>
+      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>30/08/2026 16:59</t>
+          <t>Non funziona usb</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
+        <is>
+          <t>30/08/2026 20:55</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
         <is>
           <t>angelotassi@MacBook-Air-di-Angelo.local</t>
         </is>
@@ -1045,26 +1057,30 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>IT-0101</t>
+          <t>7778238723232030230</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Iphone</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 4</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>PF4A1B2C</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>7778238723232030230</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Giuseppe sticazzi</t>
+        </is>
+      </c>
       <c r="G12" t="inlineStr">
         <is>
           <t>Site Services BAU</t>
@@ -1072,22 +1088,23 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Disponibile</t>
+          <t>Da Rispedire</t>
         </is>
       </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>Postazione reception</t>
-        </is>
-      </c>
+      <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>30/08/2026 14:58</t>
+          <t>Da rispedire a telefonia</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
+        <is>
+          <t>30/08/2026 16:59</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
         <is>
           <t>angelotassi@MacBook-Air-di-Angelo.local</t>
         </is>
@@ -1096,7 +1113,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>IT-0102</t>
+          <t>IT-0101</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1111,7 +1128,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>PF4A1B7D</t>
+          <t>PF4A1B2C</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
@@ -1131,10 +1148,15 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
+          <t>Postazione reception</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
           <t>30/08/2026 14:58</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>angelotassi@MacBook-Air-di-Angelo.local</t>
         </is>
@@ -1143,7 +1165,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>IT-0103</t>
+          <t>IT-0102</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1153,12 +1175,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 5</t>
+          <t>Lenovo ThinkPad T14 Gen 4</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>PF5K9M3E</t>
+          <t>PF4A1B7D</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
@@ -1175,17 +1197,14 @@
       </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>Batteria da sostituire</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr">
         <is>
           <t>30/08/2026 14:58</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>angelotassi@MacBook-Air-di-Angelo.local</t>
         </is>
@@ -1194,22 +1213,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>IT-0104</t>
+          <t>IT-0103</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Tablet</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Dell Latitude 7320 Detachable</t>
+          <t>Lenovo ThinkPad T14 Gen 5</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>8H2KLM3</t>
+          <t>PF5K9M3E</t>
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
@@ -1226,17 +1245,18 @@
       </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>Con tastiera e pennino</t>
-        </is>
-      </c>
+      <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
+          <t>Batteria da sostituire</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
           <t>30/08/2026 14:58</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>angelotassi@MacBook-Air-di-Angelo.local</t>
         </is>
@@ -1245,7 +1265,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>IT-0105</t>
+          <t>IT-0104</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1255,12 +1275,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Dell Latitude 7230 Rugged Extreme</t>
+          <t>Dell Latitude 7320 Detachable</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>4RT9WQ2</t>
+          <t>8H2KLM3</t>
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
@@ -1280,17 +1300,70 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
+          <t>Con tastiera e pennino</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
           <t>30/08/2026 14:58</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>IT-0105</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Tablet</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Dell Latitude 7230 Rugged Extreme</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>4RT9WQ2</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Site Services BAU</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>30/08/2026 14:58</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
         <is>
           <t>angelotassi@MacBook-Air-di-Angelo.local</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M16"/>
+  <autoFilter ref="A1:N17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Distingue meglio i tablet e chiarisce la spedizione degli iPhone
I tablet Dell passano dall'arancione all'azzurro: sul chiaro l'arancione si
confondeva con il rosso dei dispositivi in prestito.

Lo stato di un iPhone spedito diventa "Spedito al servizio telefonia" invece
del solo "Spedito", e il pulsante sulla riga dice "Conferma spedizione" invece
di "SPEDITO", cosi' e' chiaro che apre una conferma e non agisce subito.
Le colonne Stato e Prestito si allargano per contenerli.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Esempio/Inventario.xlsx
+++ b/Esempio/Inventario.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventario" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventario'!$A$1:$N$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventario'!$A$1:$N$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -442,7 +442,7 @@
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
     <col width="38" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
     <col width="24" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
@@ -1003,28 +1003,28 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>3000003843943</t>
-        </is>
-      </c>
+      <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Iphone</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Lenovo T14 gen 5</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>asdaksjhdkajsdh</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>234728342836478264</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Giovanni stepalle</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr">
         <is>
           <t>Site Services BAU</t>
@@ -1032,20 +1032,20 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Da rebuildare</t>
+          <t>Spedito</t>
         </is>
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>Non funziona usb</t>
-        </is>
-      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>30/08/2026 21:26</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr">
         <is>
-          <t>30/08/2026 20:55</t>
+          <t>30/08/2026 21:26:38</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1057,30 +1057,26 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>7778238723232030230</t>
+          <t>3000003843943</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Iphone</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>7778238723232030230</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Giuseppe sticazzi</t>
-        </is>
-      </c>
+          <t>Lenovo T14 gen 5</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>asdaksjhdkajsdh</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
           <t>Site Services BAU</t>
@@ -1088,7 +1084,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Da Rispedire</t>
+          <t>Da rebuildare</t>
         </is>
       </c>
       <c r="I12" t="inlineStr"/>
@@ -1096,12 +1092,12 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Da rispedire a telefonia</t>
+          <t>Non funziona usb</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>30/08/2026 16:59</t>
+          <t>30/08/2026 20:55</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1111,28 +1107,28 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>IT-0101</t>
-        </is>
-      </c>
+      <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Iphone</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 4</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>PF4A1B2C</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>7778238723232030230</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Giuseppe sticazzi</t>
+        </is>
+      </c>
       <c r="G13" t="inlineStr">
         <is>
           <t>Site Services BAU</t>
@@ -1140,7 +1136,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Disponibile</t>
+          <t>Da Rispedire</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>
@@ -1148,12 +1144,12 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Postazione reception</t>
+          <t>Da rispedire a telefonia</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>30/08/2026 14:58</t>
+          <t>30/08/2026 16:59</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1165,7 +1161,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>IT-0102</t>
+          <t>IT-0101</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1180,7 +1176,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>PF4A1B7D</t>
+          <t>PF4A1B2C</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
@@ -1198,7 +1194,11 @@
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Postazione reception</t>
+        </is>
+      </c>
       <c r="M14" t="inlineStr">
         <is>
           <t>30/08/2026 14:58</t>
@@ -1213,7 +1213,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>IT-0103</t>
+          <t>IT-0102</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1223,12 +1223,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 5</t>
+          <t>Lenovo ThinkPad T14 Gen 4</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>PF5K9M3E</t>
+          <t>PF4A1B7D</t>
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
@@ -1246,11 +1246,7 @@
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>Batteria da sostituire</t>
-        </is>
-      </c>
+      <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr">
         <is>
           <t>30/08/2026 14:58</t>
@@ -1265,22 +1261,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>IT-0104</t>
+          <t>IT-0103</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Tablet</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Dell Latitude 7320 Detachable</t>
+          <t>Lenovo ThinkPad T14 Gen 5</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>8H2KLM3</t>
+          <t>PF5K9M3E</t>
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
@@ -1300,7 +1296,7 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Con tastiera e pennino</t>
+          <t>Batteria da sostituire</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1317,7 +1313,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>IT-0105</t>
+          <t>IT-0104</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1327,12 +1323,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Dell Latitude 7230 Rugged Extreme</t>
+          <t>Dell Latitude 7320 Detachable</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>4RT9WQ2</t>
+          <t>8H2KLM3</t>
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
@@ -1350,7 +1346,11 @@
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Con tastiera e pennino</t>
+        </is>
+      </c>
       <c r="M17" t="inlineStr">
         <is>
           <t>30/08/2026 14:58</t>
@@ -1362,8 +1362,56 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>IT-0105</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Tablet</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Dell Latitude 7230 Rugged Extreme</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>4RT9WQ2</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Site Services BAU</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>30/08/2026 14:58</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N17"/>
+  <autoFilter ref="A1:N18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Anche l'importazione di stanza dalla pagina principale rispetta i separatori
Segnalato come bug, ed era in effetti un errore di progetto: l'opzione "Una
sola stanza" della finestra generale assegnava tutte le righe alla stanza
scelta, mentre il pulsante dentro la stanza si fidava dei separatori. Due
comportamenti diversi per la stessa operazione.

Ora la regola e' una sola, condivisa dalle due strade: se il foglio dichiara le
stanze comandano i separatori e le righe delle altre stanze si scartano; se non
le dichiara vale la stanza scelta per tutte le righe; se le dichiara ma non
comprende quella scelta non si importa niente e un avviso spiega cosa aggiungere.

Il riepilogo dice sempre quale delle tre situazioni si e' verificata.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Esempio/Inventario.xlsx
+++ b/Esempio/Inventario.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventario" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventario'!$A$1:$N$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventario'!$A$1:$N$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:N44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -437,7 +437,7 @@
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
@@ -797,7 +797,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>DR-0201</t>
+          <t>IT-BAU-101</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -807,12 +807,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 4</t>
+          <t>Lenovo ThinkPad T14 Gen 5</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>PF4B7T1J</t>
+          <t>PF5BA01</t>
         </is>
       </c>
       <c r="E7" t="inlineStr"/>
@@ -830,14 +830,10 @@
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>Scorta di emergenza - sigillato</t>
-        </is>
-      </c>
+      <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
-          <t>30/08/2026 14:58</t>
+          <t>30/08/2026 22:23:32</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -849,7 +845,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>DR-0202</t>
+          <t>IT-BAU-102</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -859,12 +855,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 5</t>
+          <t>Lenovo ThinkPad T14 Gen 4</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>PF5M2P4K</t>
+          <t>PF4BA02</t>
         </is>
       </c>
       <c r="E8" t="inlineStr"/>
@@ -884,12 +880,12 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Scorta di emergenza - sigillato</t>
+          <t>Postazione 1</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>30/08/2026 14:58</t>
+          <t>30/08/2026 22:23:32</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -901,22 +897,22 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>DR-0203</t>
+          <t>IT-BAU-103</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Tablet</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Dell Latitude 7320 Detachable</t>
+          <t>Lenovo ThinkPad T14 Gen 5</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>8H3NQR5</t>
+          <t>PF5BA03</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
@@ -934,14 +930,10 @@
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>Kit continuita' operativa</t>
-        </is>
-      </c>
+      <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr">
         <is>
-          <t>30/08/2026 14:58</t>
+          <t>30/08/2026 22:23:32</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -953,7 +945,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>IT-0106</t>
+          <t>IT-BAU-104</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -963,12 +955,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 5</t>
+          <t>Lenovo ThinkPad T14 Gen 4</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>PF5K9M8F</t>
+          <t>PF4BA04</t>
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
@@ -980,7 +972,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Disponibile</t>
+          <t>In attesa ritiro</t>
         </is>
       </c>
       <c r="I10" t="inlineStr"/>
@@ -988,12 +980,12 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Postazione kiosk 1</t>
+          <t>Batteria da sostituire</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>30/08/2026 16:13</t>
+          <t>30/08/2026 22:23:32</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1003,49 +995,45 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>IT-BAU-105</t>
+        </is>
+      </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Iphone</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>234728342836478264</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Giovanni stepalle</t>
-        </is>
-      </c>
+          <t>Lenovo ThinkPad T14 Gen 5</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>PF5BA05</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Site Services BAU</t>
+          <t>Magazzino Disaster Recovery</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Spedito</t>
+          <t>Guasto in attesa tecnico</t>
         </is>
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>30/08/2026 21:26</t>
-        </is>
-      </c>
+      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr">
         <is>
-          <t>30/08/2026 21:26:38</t>
+          <t>30/08/2026 22:23:32</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1057,7 +1045,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>3000003843943</t>
+          <t>IT-BAU-106</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1067,19 +1055,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Lenovo T14 gen 5</t>
+          <t>Lenovo ThinkPad T14 Gen 4</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>asdaksjhdkajsdh</t>
+          <t>PF4BA06</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Site Services BAU</t>
+          <t>Magazzino Disaster Recovery</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1092,12 +1080,12 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Non funziona usb</t>
+          <t>Con custodia</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>30/08/2026 20:55</t>
+          <t>30/08/2026 22:23:32</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1107,49 +1095,45 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>IT-BAU-107</t>
+        </is>
+      </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Iphone</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>7778238723232030230</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Giuseppe sticazzi</t>
-        </is>
-      </c>
+          <t>Lenovo ThinkPad T14 Gen 5</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>PF5BA07</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Site Services BAU</t>
+          <t>Magazzino Disaster Recovery</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Da Rispedire</t>
+          <t>Controllare</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>Da rispedire a telefonia</t>
-        </is>
-      </c>
+      <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr">
         <is>
-          <t>30/08/2026 16:59</t>
+          <t>30/08/2026 22:23:32</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1161,29 +1145,29 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>IT-0101</t>
+          <t>IT-BAU-108</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Tablet</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 4</t>
+          <t>Dell Latitude 7320 Detachable</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>PF4A1B2C</t>
+          <t>7HB108</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Site Services BAU</t>
+          <t>Magazzino Disaster Recovery</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1196,12 +1180,12 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Postazione reception</t>
+          <t>In verifica</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>30/08/2026 14:58</t>
+          <t>30/08/2026 22:23:32</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1213,29 +1197,29 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>IT-0102</t>
+          <t>IT-BAU-109</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Tablet</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 4</t>
+          <t>Dell Latitude 7230 Rugged Extreme</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>PF4A1B7D</t>
+          <t>8HB109</t>
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Site Services BAU</t>
+          <t>Magazzino Disaster Recovery</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1249,7 +1233,7 @@
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr">
         <is>
-          <t>30/08/2026 14:58</t>
+          <t>30/08/2026 22:23:32</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1261,29 +1245,29 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>IT-0103</t>
+          <t>IT-BAU-110</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Tablet</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 5</t>
+          <t>Dell Latitude 7320 Detachable</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>PF5K9M3E</t>
+          <t>4HB110</t>
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Site Services BAU</t>
+          <t>Magazzino Disaster Recovery</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1296,12 +1280,12 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Batteria da sostituire</t>
+          <t>Scorta</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>30/08/2026 14:58</t>
+          <t>30/08/2026 22:23:32</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1313,29 +1297,29 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>IT-0104</t>
+          <t>IT-DRC-301</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Tablet</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Dell Latitude 7320 Detachable</t>
+          <t>Lenovo ThinkPad T14 Gen 5</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>8H2KLM3</t>
+          <t>PF5DR01</t>
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Site Services BAU</t>
+          <t>Magazzino Disaster Recovery</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1346,14 +1330,10 @@
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>Con tastiera e pennino</t>
-        </is>
-      </c>
+      <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr">
         <is>
-          <t>30/08/2026 14:58</t>
+          <t>30/08/2026 22:23:32</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1365,29 +1345,29 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>IT-0105</t>
+          <t>IT-DRC-302</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Tablet</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Dell Latitude 7230 Rugged Extreme</t>
+          <t>Lenovo ThinkPad T14 Gen 4</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>4RT9WQ2</t>
+          <t>PF4DR02</t>
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Site Services BAU</t>
+          <t>Magazzino Disaster Recovery</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1398,20 +1378,1332 @@
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Postazione 1</t>
+        </is>
+      </c>
       <c r="M18" t="inlineStr">
         <is>
+          <t>30/08/2026 22:23:32</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>IT-DRC-303</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Lenovo ThinkPad T14 Gen 5</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>PF5DR03</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Magazzino Disaster Recovery</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>30/08/2026 22:23:32</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>IT-DRC-304</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Lenovo ThinkPad T14 Gen 4</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>PF4DR04</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Magazzino Disaster Recovery</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>In attesa ritiro</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Batteria da sostituire</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>30/08/2026 22:23:32</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>IT-DRC-305</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Lenovo ThinkPad T14 Gen 5</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>PF5DR05</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Magazzino Disaster Recovery</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Guasto in attesa tecnico</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>30/08/2026 22:23:32</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>IT-DRC-306</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Lenovo ThinkPad T14 Gen 4</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>PF4DR06</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Magazzino Disaster Recovery</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Da rebuildare</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Con custodia</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>30/08/2026 22:23:32</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>IT-DRC-307</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Lenovo ThinkPad T14 Gen 5</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>PF5DR07</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Magazzino Disaster Recovery</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Controllare</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>30/08/2026 22:23:32</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>IT-DRC-308</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Tablet</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Dell Latitude 7320 Detachable</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>7HD308</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Magazzino Disaster Recovery</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>In verifica</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>30/08/2026 22:23:32</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>IT-DRC-309</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Tablet</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Dell Latitude 7230 Rugged Extreme</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>8HD309</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Magazzino Disaster Recovery</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>30/08/2026 22:23:32</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>IT-DRC-310</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Tablet</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Dell Latitude 7320 Detachable</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>4HD310</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Magazzino Disaster Recovery</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Scorta</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>30/08/2026 22:23:32</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>IT-KSK-201</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Lenovo ThinkPad T14 Gen 5</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>PF5KS01</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Magazzino Disaster Recovery</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>30/08/2026 22:23:32</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>IT-KSK-202</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Lenovo ThinkPad T14 Gen 4</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>PF4KS02</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Magazzino Disaster Recovery</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Postazione 1</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>30/08/2026 22:23:32</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>IT-KSK-203</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Lenovo ThinkPad T14 Gen 5</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>PF5KS03</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Magazzino Disaster Recovery</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>30/08/2026 22:23:32</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>IT-KSK-204</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Lenovo ThinkPad T14 Gen 4</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>PF4KS04</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Magazzino Disaster Recovery</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>In attesa ritiro</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Batteria da sostituire</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>30/08/2026 22:23:32</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>IT-KSK-205</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Lenovo ThinkPad T14 Gen 5</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>PF5KS05</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Magazzino Disaster Recovery</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Guasto in attesa tecnico</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>30/08/2026 22:23:32</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>IT-KSK-206</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Lenovo ThinkPad T14 Gen 4</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>PF4KS06</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Magazzino Disaster Recovery</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Da rebuildare</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>Con custodia</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>30/08/2026 22:23:32</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>IT-KSK-207</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Lenovo ThinkPad T14 Gen 5</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>PF5KS07</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Magazzino Disaster Recovery</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Controllare</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>30/08/2026 22:23:32</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>IT-KSK-208</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Tablet</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Dell Latitude 7320 Detachable</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>7HK208</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Magazzino Disaster Recovery</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>In verifica</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>30/08/2026 22:23:32</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>IT-KSK-209</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Tablet</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Dell Latitude 7230 Rugged Extreme</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>8HK209</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Magazzino Disaster Recovery</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>30/08/2026 22:23:32</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>IT-KSK-210</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Tablet</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Dell Latitude 7320 Detachable</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>4HK210</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Magazzino Disaster Recovery</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>Scorta</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>30/08/2026 22:23:32</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr"/>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Iphone</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>234728342836478264</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Giovanni stepalle</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Site Services BAU</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Spedito al servizio telefonia</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>30/08/2026 21:26</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>30/08/2026 21:26:38</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>3000003843943</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Lenovo T14 gen 5</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>asdaksjhdkajsdh</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Site Services BAU</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Da rebuildare</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>Non funziona usb</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>30/08/2026 20:55</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr"/>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Iphone</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>7778238723232030230</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Giuseppe sticazzi</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Site Services BAU</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Da Rispedire</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Da rispedire a telefonia</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>30/08/2026 16:59</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>IT-0101</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Lenovo ThinkPad T14 Gen 4</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>PF4A1B2C</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Site Services BAU</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Postazione reception</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
           <t>30/08/2026 14:58</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr">
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>IT-0102</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Lenovo ThinkPad T14 Gen 4</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>PF4A1B7D</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Site Services BAU</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>30/08/2026 14:58</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>IT-0103</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Lenovo ThinkPad T14 Gen 5</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>PF5K9M3E</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Site Services BAU</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Batteria da sostituire</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>30/08/2026 14:58</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>IT-0104</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Tablet</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Dell Latitude 7320 Detachable</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>8H2KLM3</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Site Services BAU</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Con tastiera e pennino</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>30/08/2026 14:58</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>IT-0105</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Tablet</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Dell Latitude 7230 Rugged Extreme</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>4RT9WQ2</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Site Services BAU</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>30/08/2026 14:58</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
         <is>
           <t>angelotassi@MacBook-Air-di-Angelo.local</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N18"/>
+  <autoFilter ref="A1:N44"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
L'esportazione chiede ambito e forma, come l'importazione
Esporta xls... apre prima una finestra con la stessa struttura di quella di
importazione: tutto l'inventario o una sola stanza, e - per l'inventario intero
- un unico elenco, un foglio per stanza o un file separato per stanza.

Corretto il difetto segnalato: scegliendo un foglio per stanza il codice
toglieva la colonna Stanza e non scriveva nessun titolo, cosi' il foglio non
diceva a quale stanza appartenesse. Ora ogni foglio porta il nome della stanza
in A1, la data e il conteggio, e conserva la colonna Stanza.

L'esportazione partiva inoltre dalla vista corrente, filtri compresi: e' il
motivo per cui usciva un foglio con dieci righe. Ora esporta quello che si e'
scelto nella finestra.

La lettura dei file scorre tutti i fogli invece del solo primo, e usa il nome
del foglio come riga-separatore: cosi' un'esportazione con un foglio per stanza
si puo' reimportare.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Esempio/Inventario.xlsx
+++ b/Esempio/Inventario.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventario" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventario'!$A$1:$N$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventario'!$A$1:$N$33</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N44"/>
+  <dimension ref="A1:N33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -521,7 +521,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>30000005678450</t>
+          <t>IT-KSK-201</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -531,12 +531,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>t14 gen 4</t>
+          <t>Lenovo ThinkPad T14 Gen 5</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>agsdad76df</t>
+          <t>PF5KS01</t>
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
@@ -548,28 +548,16 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Non disponibile</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Francesco Ricci</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>30/08/2026 17:00</t>
-        </is>
-      </c>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>test3</t>
-        </is>
-      </c>
+      <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>30/08/2026 17:00</t>
+          <t>30/08/2026 22:31:46</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -581,7 +569,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>IT-0107</t>
+          <t>IT-KSK-202</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -596,7 +584,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>PF4A2C1G</t>
+          <t>PF4KS02</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
@@ -608,24 +596,20 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Non disponibile</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Marco Bianchi</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>30/08/2026 14:58</t>
-        </is>
-      </c>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Postazione 1</t>
+        </is>
+      </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>30/08/2026 14:58</t>
+          <t>30/08/2026 22:31:46</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -637,7 +621,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>IT-0108</t>
+          <t>IT-KSK-203</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -652,7 +636,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>PF5L4N2H</t>
+          <t>PF5KS03</t>
         </is>
       </c>
       <c r="E4" t="inlineStr"/>
@@ -670,14 +654,10 @@
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Postazione kiosk 2</t>
-        </is>
-      </c>
+      <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>30/08/2026 14:58</t>
+          <t>30/08/2026 22:31:46</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -689,22 +669,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>IT-0109</t>
+          <t>IT-KSK-204</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Tablet</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Dell Latitude 7320 Detachable</t>
+          <t>Lenovo ThinkPad T14 Gen 4</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>8H2KLP9</t>
+          <t>PF4KS04</t>
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
@@ -716,16 +696,20 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Disponibile</t>
+          <t>In attesa ritiro</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Batteria da sostituire</t>
+        </is>
+      </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>30/08/2026 14:58</t>
+          <t>30/08/2026 22:31:46</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -737,22 +721,22 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>IT-0110</t>
+          <t>IT-KSK-205</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Tablet</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Dell Latitude 7230 Rugged Extreme</t>
+          <t>Lenovo ThinkPad T14 Gen 5</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>4RT9WX7</t>
+          <t>PF5KS05</t>
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
@@ -764,28 +748,16 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Non disponibile</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Elena Rossi</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>30/08/2026 14:58</t>
-        </is>
-      </c>
+          <t>Guasto in attesa tecnico</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>Con custodia rinforzata</t>
-        </is>
-      </c>
+      <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr">
         <is>
-          <t>30/08/2026 14:58</t>
+          <t>30/08/2026 22:31:46</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -797,7 +769,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>IT-BAU-101</t>
+          <t>IT-KSK-206</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -807,33 +779,37 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 5</t>
+          <t>Lenovo ThinkPad T14 Gen 4</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>PF5BA01</t>
+          <t>PF4KS06</t>
         </is>
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Magazzino Disaster Recovery</t>
+          <t>Digital Kiosk</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Disponibile</t>
+          <t>Da rebuildare</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Con custodia</t>
+        </is>
+      </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>30/08/2026 22:23:32</t>
+          <t>30/08/2026 22:31:46</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -845,7 +821,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>IT-BAU-102</t>
+          <t>IT-KSK-207</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -855,37 +831,33 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 4</t>
+          <t>Lenovo ThinkPad T14 Gen 5</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>PF4BA02</t>
+          <t>PF5KS07</t>
         </is>
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Magazzino Disaster Recovery</t>
+          <t>Digital Kiosk</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Disponibile</t>
+          <t>Controllare</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>Postazione 1</t>
-        </is>
-      </c>
+      <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
-          <t>30/08/2026 22:23:32</t>
+          <t>30/08/2026 22:31:46</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -897,29 +869,29 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>IT-BAU-103</t>
+          <t>IT-KSK-208</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Tablet</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 5</t>
+          <t>Dell Latitude 7320 Detachable</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>PF5BA03</t>
+          <t>7HK208</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Magazzino Disaster Recovery</t>
+          <t>Digital Kiosk</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -930,10 +902,14 @@
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>In verifica</t>
+        </is>
+      </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>30/08/2026 22:23:32</t>
+          <t>30/08/2026 22:31:46</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -945,47 +921,43 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>IT-BAU-104</t>
+          <t>IT-KSK-209</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Tablet</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 4</t>
+          <t>Dell Latitude 7230 Rugged Extreme</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>PF4BA04</t>
+          <t>8HK209</t>
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Magazzino Disaster Recovery</t>
+          <t>Digital Kiosk</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>In attesa ritiro</t>
+          <t>Disponibile</t>
         </is>
       </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>Batteria da sostituire</t>
-        </is>
-      </c>
+      <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr">
         <is>
-          <t>30/08/2026 22:23:32</t>
+          <t>30/08/2026 22:31:46</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -997,43 +969,47 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>IT-BAU-105</t>
+          <t>IT-KSK-210</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Tablet</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 5</t>
+          <t>Dell Latitude 7320 Detachable</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>PF5BA05</t>
+          <t>4HK210</t>
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Magazzino Disaster Recovery</t>
+          <t>Digital Kiosk</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Guasto in attesa tecnico</t>
+          <t>Disponibile</t>
         </is>
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Scorta</t>
+        </is>
+      </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>30/08/2026 22:23:32</t>
+          <t>30/08/2026 22:31:46</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1045,7 +1021,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>IT-BAU-106</t>
+          <t>IT-DRC-301</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1055,12 +1031,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 4</t>
+          <t>Lenovo ThinkPad T14 Gen 5</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>PF4BA06</t>
+          <t>PF5DR01</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
@@ -1072,20 +1048,16 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Da rebuildare</t>
+          <t>Disponibile</t>
         </is>
       </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>Con custodia</t>
-        </is>
-      </c>
+      <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr">
         <is>
-          <t>30/08/2026 22:23:32</t>
+          <t>30/08/2026 22:31:46</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1097,7 +1069,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>IT-BAU-107</t>
+          <t>IT-DRC-302</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1107,12 +1079,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 5</t>
+          <t>Lenovo ThinkPad T14 Gen 4</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>PF5BA07</t>
+          <t>PF4DR02</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
@@ -1124,16 +1096,20 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Controllare</t>
+          <t>Disponibile</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Postazione 1</t>
+        </is>
+      </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>30/08/2026 22:23:32</t>
+          <t>30/08/2026 22:31:46</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1145,22 +1121,22 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>IT-BAU-108</t>
+          <t>IT-DRC-303</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Tablet</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Dell Latitude 7320 Detachable</t>
+          <t>Lenovo ThinkPad T14 Gen 5</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>7HB108</t>
+          <t>PF5DR03</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
@@ -1178,14 +1154,10 @@
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>In verifica</t>
-        </is>
-      </c>
+      <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr">
         <is>
-          <t>30/08/2026 22:23:32</t>
+          <t>30/08/2026 22:31:46</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1197,22 +1169,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>IT-BAU-109</t>
+          <t>IT-DRC-304</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Tablet</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Dell Latitude 7230 Rugged Extreme</t>
+          <t>Lenovo ThinkPad T14 Gen 4</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>8HB109</t>
+          <t>PF4DR04</t>
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
@@ -1224,16 +1196,20 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Disponibile</t>
+          <t>In attesa ritiro</t>
         </is>
       </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Batteria da sostituire</t>
+        </is>
+      </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>30/08/2026 22:23:32</t>
+          <t>30/08/2026 22:31:46</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1245,22 +1221,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>IT-BAU-110</t>
+          <t>IT-DRC-305</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Tablet</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Dell Latitude 7320 Detachable</t>
+          <t>Lenovo ThinkPad T14 Gen 5</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>4HB110</t>
+          <t>PF5DR05</t>
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
@@ -1272,20 +1248,16 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Disponibile</t>
+          <t>Guasto in attesa tecnico</t>
         </is>
       </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>Scorta</t>
-        </is>
-      </c>
+      <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr">
         <is>
-          <t>30/08/2026 22:23:32</t>
+          <t>30/08/2026 22:31:46</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1297,7 +1269,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>IT-DRC-301</t>
+          <t>IT-DRC-306</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1307,12 +1279,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 5</t>
+          <t>Lenovo ThinkPad T14 Gen 4</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>PF5DR01</t>
+          <t>PF4DR06</t>
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
@@ -1324,16 +1296,20 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Disponibile</t>
+          <t>Da rebuildare</t>
         </is>
       </c>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Con custodia</t>
+        </is>
+      </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>30/08/2026 22:23:32</t>
+          <t>30/08/2026 22:31:46</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1345,7 +1321,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>IT-DRC-302</t>
+          <t>IT-DRC-307</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1355,12 +1331,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 4</t>
+          <t>Lenovo ThinkPad T14 Gen 5</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>PF4DR02</t>
+          <t>PF5DR07</t>
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
@@ -1372,20 +1348,16 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Disponibile</t>
+          <t>Controllare</t>
         </is>
       </c>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>Postazione 1</t>
-        </is>
-      </c>
+      <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr">
         <is>
-          <t>30/08/2026 22:23:32</t>
+          <t>30/08/2026 22:31:46</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1397,22 +1369,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>IT-DRC-303</t>
+          <t>IT-DRC-308</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Tablet</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 5</t>
+          <t>Dell Latitude 7320 Detachable</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>PF5DR03</t>
+          <t>7HD308</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
@@ -1430,10 +1402,14 @@
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>In verifica</t>
+        </is>
+      </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>30/08/2026 22:23:32</t>
+          <t>30/08/2026 22:31:46</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1445,22 +1421,22 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>IT-DRC-304</t>
+          <t>IT-DRC-309</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Tablet</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 4</t>
+          <t>Dell Latitude 7230 Rugged Extreme</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>PF4DR04</t>
+          <t>8HD309</t>
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
@@ -1472,20 +1448,16 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>In attesa ritiro</t>
+          <t>Disponibile</t>
         </is>
       </c>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>Batteria da sostituire</t>
-        </is>
-      </c>
+      <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr">
         <is>
-          <t>30/08/2026 22:23:32</t>
+          <t>30/08/2026 22:31:46</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -1497,22 +1469,22 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>IT-DRC-305</t>
+          <t>IT-DRC-310</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Tablet</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 5</t>
+          <t>Dell Latitude 7320 Detachable</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>PF5DR05</t>
+          <t>4HD310</t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
@@ -1524,16 +1496,20 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Guasto in attesa tecnico</t>
+          <t>Disponibile</t>
         </is>
       </c>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Scorta</t>
+        </is>
+      </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>30/08/2026 22:23:32</t>
+          <t>30/08/2026 22:31:46</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -1543,49 +1519,49 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>IT-DRC-306</t>
-        </is>
-      </c>
+      <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Iphone</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 4</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>PF4DR06</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>234728342836478264</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Giovanni stepalle</t>
+        </is>
+      </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Magazzino Disaster Recovery</t>
+          <t>Site Services BAU</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Da rebuildare</t>
+          <t>Spedito al servizio telefonia</t>
         </is>
       </c>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>Con custodia</t>
-        </is>
-      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>30/08/2026 21:26</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr">
         <is>
-          <t>30/08/2026 22:23:32</t>
+          <t>30/08/2026 21:26:38</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -1595,45 +1571,49 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>IT-DRC-307</t>
-        </is>
-      </c>
+      <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Iphone</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 5</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>PF5DR07</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>7778238723232030230</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Giuseppe sticazzi</t>
+        </is>
+      </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Magazzino Disaster Recovery</t>
+          <t>Site Services BAU</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Controllare</t>
+          <t>Da Rispedire</t>
         </is>
       </c>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Da rispedire a telefonia</t>
+        </is>
+      </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>30/08/2026 22:23:32</t>
+          <t>30/08/2026 16:59</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -1645,29 +1625,29 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>IT-DRC-308</t>
+          <t>IT-BAU-101</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Tablet</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Dell Latitude 7320 Detachable</t>
+          <t>Lenovo ThinkPad T14 Gen 5</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>7HD308</t>
+          <t>PF5BA01</t>
         </is>
       </c>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Magazzino Disaster Recovery</t>
+          <t>Site Services BAU</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1678,14 +1658,10 @@
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>In verifica</t>
-        </is>
-      </c>
+      <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr">
         <is>
-          <t>30/08/2026 22:23:32</t>
+          <t>30/08/2026 22:31:46</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -1697,29 +1673,29 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>IT-DRC-309</t>
+          <t>IT-BAU-102</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Tablet</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Dell Latitude 7230 Rugged Extreme</t>
+          <t>Lenovo ThinkPad T14 Gen 4</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>8HD309</t>
+          <t>PF4BA02</t>
         </is>
       </c>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Magazzino Disaster Recovery</t>
+          <t>Site Services BAU</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1730,10 +1706,14 @@
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Postazione 1</t>
+        </is>
+      </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>30/08/2026 22:23:32</t>
+          <t>30/08/2026 22:31:46</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -1745,29 +1725,29 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>IT-DRC-310</t>
+          <t>IT-BAU-103</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Tablet</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Dell Latitude 7320 Detachable</t>
+          <t>Lenovo ThinkPad T14 Gen 5</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>4HD310</t>
+          <t>PF5BA03</t>
         </is>
       </c>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Magazzino Disaster Recovery</t>
+          <t>Site Services BAU</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1778,14 +1758,10 @@
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>Scorta</t>
-        </is>
-      </c>
+      <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr">
         <is>
-          <t>30/08/2026 22:23:32</t>
+          <t>30/08/2026 22:31:46</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -1797,7 +1773,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>IT-KSK-201</t>
+          <t>IT-BAU-104</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1807,33 +1783,37 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 5</t>
+          <t>Lenovo ThinkPad T14 Gen 4</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>PF5KS01</t>
+          <t>PF4BA04</t>
         </is>
       </c>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Magazzino Disaster Recovery</t>
+          <t>Site Services BAU</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Disponibile</t>
+          <t>In attesa ritiro</t>
         </is>
       </c>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Batteria da sostituire</t>
+        </is>
+      </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>30/08/2026 22:23:32</t>
+          <t>30/08/2026 22:31:46</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -1845,7 +1825,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>IT-KSK-202</t>
+          <t>IT-BAU-105</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1855,37 +1835,33 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 4</t>
+          <t>Lenovo ThinkPad T14 Gen 5</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>PF4KS02</t>
+          <t>PF5BA05</t>
         </is>
       </c>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Magazzino Disaster Recovery</t>
+          <t>Site Services BAU</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Disponibile</t>
+          <t>Guasto in attesa tecnico</t>
         </is>
       </c>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>Postazione 1</t>
-        </is>
-      </c>
+      <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr">
         <is>
-          <t>30/08/2026 22:23:32</t>
+          <t>30/08/2026 22:31:46</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -1897,7 +1873,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>IT-KSK-203</t>
+          <t>IT-BAU-106</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1907,33 +1883,37 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 5</t>
+          <t>Lenovo ThinkPad T14 Gen 4</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>PF5KS03</t>
+          <t>PF4BA06</t>
         </is>
       </c>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Magazzino Disaster Recovery</t>
+          <t>Site Services BAU</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Disponibile</t>
+          <t>Da rebuildare</t>
         </is>
       </c>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>Con custodia</t>
+        </is>
+      </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>30/08/2026 22:23:32</t>
+          <t>30/08/2026 22:31:46</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -1945,7 +1925,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>IT-KSK-204</t>
+          <t>IT-BAU-107</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1955,37 +1935,33 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 4</t>
+          <t>Lenovo ThinkPad T14 Gen 5</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>PF4KS04</t>
+          <t>PF5BA07</t>
         </is>
       </c>
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Magazzino Disaster Recovery</t>
+          <t>Site Services BAU</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>In attesa ritiro</t>
+          <t>Controllare</t>
         </is>
       </c>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>Batteria da sostituire</t>
-        </is>
-      </c>
+      <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr">
         <is>
-          <t>30/08/2026 22:23:32</t>
+          <t>30/08/2026 22:31:46</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -1997,43 +1973,47 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>IT-KSK-205</t>
+          <t>IT-BAU-108</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Tablet</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 5</t>
+          <t>Dell Latitude 7320 Detachable</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>PF5KS05</t>
+          <t>7HB108</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Magazzino Disaster Recovery</t>
+          <t>Site Services BAU</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Guasto in attesa tecnico</t>
+          <t>Disponibile</t>
         </is>
       </c>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>In verifica</t>
+        </is>
+      </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>30/08/2026 22:23:32</t>
+          <t>30/08/2026 22:31:46</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -2045,47 +2025,43 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>IT-KSK-206</t>
+          <t>IT-BAU-109</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Tablet</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 4</t>
+          <t>Dell Latitude 7230 Rugged Extreme</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>PF4KS06</t>
+          <t>8HB109</t>
         </is>
       </c>
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Magazzino Disaster Recovery</t>
+          <t>Site Services BAU</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Da rebuildare</t>
+          <t>Disponibile</t>
         </is>
       </c>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>Con custodia</t>
-        </is>
-      </c>
+      <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr">
         <is>
-          <t>30/08/2026 22:23:32</t>
+          <t>30/08/2026 22:31:46</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -2097,43 +2073,47 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>IT-KSK-207</t>
+          <t>IT-BAU-110</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Tablet</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 5</t>
+          <t>Dell Latitude 7320 Detachable</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>PF5KS07</t>
+          <t>4HB110</t>
         </is>
       </c>
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Magazzino Disaster Recovery</t>
+          <t>Site Services BAU</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Controllare</t>
+          <t>Disponibile</t>
         </is>
       </c>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Scorta</t>
+        </is>
+      </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>30/08/2026 22:23:32</t>
+          <t>30/08/2026 22:31:46</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -2142,568 +2122,8 @@
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>IT-KSK-208</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Tablet</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Dell Latitude 7320 Detachable</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>7HK208</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>Magazzino Disaster Recovery</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>In verifica</t>
-        </is>
-      </c>
-      <c r="M34" t="inlineStr">
-        <is>
-          <t>30/08/2026 22:23:32</t>
-        </is>
-      </c>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>IT-KSK-209</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Tablet</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Dell Latitude 7230 Rugged Extreme</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>8HK209</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>Magazzino Disaster Recovery</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>30/08/2026 22:23:32</t>
-        </is>
-      </c>
-      <c r="N35" t="inlineStr">
-        <is>
-          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>IT-KSK-210</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Tablet</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Dell Latitude 7320 Detachable</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>4HK210</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>Magazzino Disaster Recovery</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>Scorta</t>
-        </is>
-      </c>
-      <c r="M36" t="inlineStr">
-        <is>
-          <t>30/08/2026 22:23:32</t>
-        </is>
-      </c>
-      <c r="N36" t="inlineStr">
-        <is>
-          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr"/>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Iphone</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>234728342836478264</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>Giovanni stepalle</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>Site Services BAU</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>Spedito al servizio telefonia</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>30/08/2026 21:26</t>
-        </is>
-      </c>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr">
-        <is>
-          <t>30/08/2026 21:26:38</t>
-        </is>
-      </c>
-      <c r="N37" t="inlineStr">
-        <is>
-          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>3000003843943</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Laptop</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Lenovo T14 gen 5</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>asdaksjhdkajsdh</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>Site Services BAU</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>Da rebuildare</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>Non funziona usb</t>
-        </is>
-      </c>
-      <c r="M38" t="inlineStr">
-        <is>
-          <t>30/08/2026 20:55</t>
-        </is>
-      </c>
-      <c r="N38" t="inlineStr">
-        <is>
-          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr"/>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Iphone</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>7778238723232030230</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>Giuseppe sticazzi</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>Site Services BAU</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>Da Rispedire</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr">
-        <is>
-          <t>Da rispedire a telefonia</t>
-        </is>
-      </c>
-      <c r="M39" t="inlineStr">
-        <is>
-          <t>30/08/2026 16:59</t>
-        </is>
-      </c>
-      <c r="N39" t="inlineStr">
-        <is>
-          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>IT-0101</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Laptop</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>Lenovo ThinkPad T14 Gen 4</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>PF4A1B2C</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>Site Services BAU</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr">
-        <is>
-          <t>Postazione reception</t>
-        </is>
-      </c>
-      <c r="M40" t="inlineStr">
-        <is>
-          <t>30/08/2026 14:58</t>
-        </is>
-      </c>
-      <c r="N40" t="inlineStr">
-        <is>
-          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>IT-0102</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Laptop</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Lenovo ThinkPad T14 Gen 4</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>PF4A1B7D</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>Site Services BAU</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr">
-        <is>
-          <t>30/08/2026 14:58</t>
-        </is>
-      </c>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>IT-0103</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Laptop</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Lenovo ThinkPad T14 Gen 5</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>PF5K9M3E</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>Site Services BAU</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>Batteria da sostituire</t>
-        </is>
-      </c>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t>30/08/2026 14:58</t>
-        </is>
-      </c>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>IT-0104</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Tablet</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Dell Latitude 7320 Detachable</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>8H2KLM3</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr"/>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>Site Services BAU</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>Con tastiera e pennino</t>
-        </is>
-      </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>30/08/2026 14:58</t>
-        </is>
-      </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>IT-0105</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Tablet</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>Dell Latitude 7230 Rugged Extreme</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>4RT9WQ2</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>Site Services BAU</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>30/08/2026 14:58</t>
-        </is>
-      </c>
-      <c r="N44" t="inlineStr">
-        <is>
-          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:N44"/>
+  <autoFilter ref="A1:N33"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Allinea la documentazione e isola i test dalla configurazione reale
La pagina del progetto aveva tre schede in meno nella versione italiana e una
in meno in quella inglese: ora ne hanno undici ciascuna, con lo stesso
contenuto. Entrambe rimandano alla guida al formato dei file, dal pulsante in
cima e dalla scheda su Excel.

I due README dicevano che la lingua si cambia dalle impostazioni, mentre la
tendina e' anche nell'intestazione. Le istruzioni di collaudo guadagnano un nono
scenario sul cambio di lingua e sull'esportazione in inglese, e rimandano alla
guida per chi prepara un file suo.

Le suite non leggono ne' scrivono piu' inventario_percorso.json: la preferenza
di lingua salvata sul computer faceva fallire dieci test su diciotto a seconda
di come era rimasta, e i test la sovrascrivevano a loro volta.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Esempio/Inventario.xlsx
+++ b/Esempio/Inventario.xlsx
@@ -1093,7 +1093,7 @@
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr">
         <is>
-          <t>30/08/2026 23:34:23</t>
+          <t>30/08/2026 23:55:35</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1145,7 +1145,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>30/08/2026 23:34:23</t>
+          <t>30/08/2026 23:55:35</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1193,7 +1193,7 @@
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr">
         <is>
-          <t>30/08/2026 23:34:23</t>
+          <t>30/08/2026 23:55:35</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1245,7 +1245,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>30/08/2026 23:34:23</t>
+          <t>30/08/2026 23:55:35</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1293,7 +1293,7 @@
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr">
         <is>
-          <t>30/08/2026 23:34:23</t>
+          <t>30/08/2026 23:55:35</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>30/08/2026 23:34:23</t>
+          <t>30/08/2026 23:55:35</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1393,7 +1393,7 @@
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr">
         <is>
-          <t>30/08/2026 23:34:23</t>
+          <t>30/08/2026 23:55:35</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>30/08/2026 23:34:23</t>
+          <t>30/08/2026 23:55:35</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1493,7 +1493,7 @@
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr">
         <is>
-          <t>30/08/2026 23:34:23</t>
+          <t>30/08/2026 23:55:35</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -1545,7 +1545,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>30/08/2026 23:34:23</t>
+          <t>30/08/2026 23:55:35</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">

</xml_diff>

<commit_message>
Separa l'inventario vero dai dati dimostrativi
La configurazione locale puntava a Esempio/Inventario.xlsx: l'inventario
dell'utente viveva dentro il repository, dove le prove lo sovrascrivevano e da
dove sarebbe finito in un repository pubblico. I dati veri sono stati spostati
fuori, e il percorso memorizzato ora punta li'.

Esempio/ torna a contenere i tredici dispositivi finti che dovrebbe avere, con i
due prestiti in corso nel Digital Kiosk, e si rigenera con
tests/genera_esempio.py invece di dipendere da quello che c'era prima.

I due README spiegano dove tenere l'inventario vero e come cambiare il percorso.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Esempio/Inventario.xlsx
+++ b/Esempio/Inventario.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventario" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventario'!$A$1:$N$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventario'!$A$1:$N$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N21"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -521,7 +521,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>30000005678450</t>
+          <t>IT-0106</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -531,12 +531,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>t14 gen 4</t>
+          <t>Lenovo ThinkPad T14 Gen 5</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>agsdad76df</t>
+          <t>PF5K9M8F</t>
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
@@ -548,28 +548,20 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Non disponibile</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Francesco Ricci</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>30/08/2026 17:00</t>
-        </is>
-      </c>
+          <t>Disponibile</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
-          <t>test3</t>
+          <t>Postazione kiosk 1</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>30/08/2026 17:00</t>
+          <t>31/08/2026 00:01:50</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -618,14 +610,14 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>30/08/2026 14:58</t>
+          <t>31/08/2026 00:01</t>
         </is>
       </c>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>30/08/2026 14:58</t>
+          <t>31/08/2026 00:01:51</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -677,7 +669,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>30/08/2026 14:58</t>
+          <t>31/08/2026 00:01:50</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -725,7 +717,7 @@
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>30/08/2026 14:58</t>
+          <t>31/08/2026 00:01:50</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -774,18 +766,18 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>30/08/2026 14:58</t>
+          <t>31/08/2026 00:01</t>
         </is>
       </c>
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Con custodia rinforzata</t>
+          <t>Con custodia</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>30/08/2026 14:58</t>
+          <t>31/08/2026 00:01:51</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -832,12 +824,12 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Scorta di emergenza - sigillato</t>
+          <t>Scorta sigillata</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>30/08/2026 14:58</t>
+          <t>31/08/2026 00:01:50</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -884,12 +876,12 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Scorta di emergenza - sigillato</t>
+          <t>Scorta sigillata</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>30/08/2026 14:58</t>
+          <t>31/08/2026 00:01:50</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -941,7 +933,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>30/08/2026 14:58</t>
+          <t>31/08/2026 00:01:51</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -953,7 +945,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>IT-0106</t>
+          <t>IT-0101</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -963,19 +955,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 5</t>
+          <t>Lenovo ThinkPad T14 Gen 4</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>PF5K9M8F</t>
+          <t>PF4A1B2C</t>
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Magazzino Disaster Recovery</t>
+          <t>Site Services BAU</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -988,12 +980,12 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Postazione kiosk 1</t>
+          <t>Postazione reception</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>30/08/2026 16:13</t>
+          <t>31/08/2026 00:01:50</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1003,28 +995,28 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>IT-0102</t>
+        </is>
+      </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Iphone</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>7778238723232030230</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Giuseppe sticazzi</t>
-        </is>
-      </c>
+          <t>Lenovo ThinkPad T14 Gen 4</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>PF4A1B7D</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>Site Services BAU</t>
@@ -1032,20 +1024,16 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Da Rispedire</t>
+          <t>Disponibile</t>
         </is>
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>Da rispedire a telefonia</t>
-        </is>
-      </c>
+      <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr">
         <is>
-          <t>30/08/2026 16:59</t>
+          <t>31/08/2026 00:01:50</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1057,7 +1045,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>IT-BAU-101</t>
+          <t>IT-0103</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1072,7 +1060,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>PF5BA01</t>
+          <t>PF5K9M3E</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
@@ -1090,10 +1078,14 @@
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Batteria da sostituire</t>
+        </is>
+      </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>30/08/2026 23:55:35</t>
+          <t>31/08/2026 00:01:50</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1105,22 +1097,22 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>IT-BAU-102</t>
+          <t>IT-0104</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Tablet</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 4</t>
+          <t>Dell Latitude 7320 Detachable</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>PF4BA02</t>
+          <t>8H2KLM3</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
@@ -1140,12 +1132,12 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Postazione 1</t>
+          <t>Con tastiera e pennino</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>30/08/2026 23:55:35</t>
+          <t>31/08/2026 00:01:50</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1157,22 +1149,22 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>IT-BAU-103</t>
+          <t>IT-0105</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Tablet</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14 Gen 5</t>
+          <t>Dell Latitude 7230 Rugged Extreme</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>PF5BA03</t>
+          <t>4RT9WQ2</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
@@ -1193,7 +1185,7 @@
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr">
         <is>
-          <t>30/08/2026 23:55:35</t>
+          <t>31/08/2026 00:01:50</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1202,360 +1194,8 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>IT-BAU-104</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Laptop</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Lenovo ThinkPad T14 Gen 4</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>PF4BA04</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Site Services BAU</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>In attesa ritiro</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>Batteria da sostituire</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>30/08/2026 23:55:35</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>IT-BAU-105</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Laptop</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Lenovo ThinkPad T14 Gen 5</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>PF5BA05</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Site Services BAU</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Guasto in attesa tecnico</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>30/08/2026 23:55:35</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>IT-BAU-106</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Laptop</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Lenovo ThinkPad T14 Gen 4</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>PF4BA06</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Site Services BAU</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>Da rebuildare</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>Con custodia</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>30/08/2026 23:55:35</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>IT-BAU-107</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Laptop</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Lenovo ThinkPad T14 Gen 5</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>PF5BA07</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Site Services BAU</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>Controllare</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>30/08/2026 23:55:35</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>IT-BAU-108</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Tablet</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Dell Latitude 7320 Detachable</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>7HB108</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Site Services BAU</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>In verifica</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>30/08/2026 23:55:35</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>IT-BAU-109</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Tablet</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Dell Latitude 7230 Rugged Extreme</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>8HB109</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Site Services BAU</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>30/08/2026 23:55:35</t>
-        </is>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>IT-BAU-110</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Tablet</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Dell Latitude 7320 Detachable</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>4HB110</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Site Services BAU</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>Disponibile</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>Scorta</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>30/08/2026 23:55:35</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>angelotassi@MacBook-Air-di-Angelo.local</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:N21"/>
+  <autoFilter ref="A1:N14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>